<commit_message>
Tried adding better implementation temperature and tried adding rock type mapping for SOM
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Zwischenstände/SVZ-CHILE_Datenbank/after_conversion_chile_mapped_readable.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Zwischenstände/SVZ-CHILE_Datenbank/after_conversion_chile_mapped_readable.xlsx
@@ -807,13 +807,16 @@
         <v>2.4</v>
       </c>
       <c r="L4">
-        <v>16.63112752551153</v>
+        <v>18.52061952917278</v>
       </c>
       <c r="N4">
-        <v>1.157036419113215</v>
+        <v>2.527211125957812</v>
+      </c>
+      <c r="O4">
+        <v>2.139477473770829</v>
       </c>
       <c r="P4">
-        <v>1.297469933629422</v>
+        <v>2.028544338539847</v>
       </c>
       <c r="Q4">
         <v>0.3334273624823695</v>
@@ -822,10 +825,10 @@
         <v>9.179575265459087</v>
       </c>
       <c r="S4">
-        <v>0.9521967720365538</v>
+        <v>0</v>
       </c>
       <c r="U4">
-        <v>2.079374295046076</v>
+        <v>0.6803364852180274</v>
       </c>
       <c r="V4">
         <v>1632.047477744807</v>
@@ -910,13 +913,16 @@
         <v>2.7</v>
       </c>
       <c r="L6">
-        <v>27.5523865636992</v>
+        <v>28.31882445972851</v>
       </c>
       <c r="N6">
-        <v>0.543720121763729</v>
+        <v>0.9960952630711514</v>
+      </c>
+      <c r="O6">
+        <v>0.9956799012548858</v>
       </c>
       <c r="P6">
-        <v>0.6038225460352312</v>
+        <v>0.8857727431508557</v>
       </c>
       <c r="Q6">
         <v>0.0062059238363892</v>
@@ -925,10 +931,10 @@
         <v>23.50614199458672</v>
       </c>
       <c r="S6">
-        <v>0.3753064729713783</v>
+        <v>0</v>
       </c>
       <c r="U6">
-        <v>0.9079678656105252</v>
+        <v>0.3197069949332835</v>
       </c>
       <c r="V6">
         <v>1609.221638895229</v>
@@ -960,13 +966,16 @@
         <v>3.6</v>
       </c>
       <c r="L7">
-        <v>6.907230042490595</v>
+        <v>7.461714377447538</v>
       </c>
       <c r="N7">
-        <v>0.5393703607896191</v>
+        <v>1.204883789828423</v>
+      </c>
+      <c r="O7">
+        <v>0.0987451141740382</v>
       </c>
       <c r="P7">
-        <v>0.0598832277059733</v>
+        <v>0.5214831079395179</v>
       </c>
       <c r="Q7">
         <v>0.0090267983074753</v>
@@ -975,10 +984,10 @@
         <v>4.315219654382677</v>
       </c>
       <c r="S7">
-        <v>0.4539733319348114</v>
+        <v>0</v>
       </c>
       <c r="U7">
-        <v>0.53455009552845</v>
+        <v>0.3171493389738172</v>
       </c>
       <c r="V7">
         <v>995.2065738415886</v>

</xml_diff>